<commit_message>
data: preserve eligibility using compatible shared strings
</commit_message>
<xml_diff>
--- a/fuel_cost_chungcheong.xlsx
+++ b/fuel_cost_chungcheong.xlsx
@@ -9782,10 +9782,8 @@
         <f t="shared" si="6"/>
         <v>90260</v>
       </c>
-      <c r="Q51" s="12" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
+      <c r="Q51" s="12" t="s">
+        <v>61</v>
       </c>
       <c r="R51" s="13">
         <f t="shared" si="7"/>
@@ -9946,10 +9944,8 @@
         <f t="shared" si="6"/>
         <v>90260</v>
       </c>
-      <c r="Q53" s="12" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
+      <c r="Q53" s="12" t="s">
+        <v>61</v>
       </c>
       <c r="R53" s="13">
         <f t="shared" si="7"/>
@@ -11310,10 +11306,8 @@
         <f t="shared" si="6"/>
         <v>90950</v>
       </c>
-      <c r="Q70" s="12" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
+      <c r="Q70" s="12" t="s">
+        <v>61</v>
       </c>
       <c r="R70" s="13">
         <f t="shared" si="7"/>
@@ -11394,10 +11388,8 @@
         <f t="shared" si="6"/>
         <v>90975</v>
       </c>
-      <c r="Q71" s="12" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
+      <c r="Q71" s="12" t="s">
+        <v>61</v>
       </c>
       <c r="R71" s="13">
         <f t="shared" si="7"/>
@@ -11718,10 +11710,8 @@
         <f t="shared" si="6"/>
         <v>91105</v>
       </c>
-      <c r="Q75" s="12" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
+      <c r="Q75" s="12" t="s">
+        <v>61</v>
       </c>
       <c r="R75" s="13">
         <f t="shared" si="7"/>
@@ -12442,10 +12432,8 @@
         <f t="shared" si="19"/>
         <v>91485</v>
       </c>
-      <c r="Q84" s="12" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
+      <c r="Q84" s="12" t="s">
+        <v>61</v>
       </c>
       <c r="R84" s="13">
         <f t="shared" si="20"/>
@@ -14206,10 +14194,8 @@
         <f t="shared" si="19"/>
         <v>92010</v>
       </c>
-      <c r="Q106" s="12" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
+      <c r="Q106" s="12" t="s">
+        <v>61</v>
       </c>
       <c r="R106" s="13">
         <f t="shared" si="20"/>
@@ -37422,10 +37408,8 @@
         <f t="shared" ref="P399:P462" si="84">IF($B$10=0,"",IFERROR(IF($B$4&gt;0,IF($L399="",1/0,$L399*$B$4),0)+IF($B$5&gt;0,IF($M399="",1/0,$M399*$B$5),0)+IF($B$6&gt;0,IF($N399="",1/0,$N399*$B$6),0),""))</f>
         <v/>
       </c>
-      <c r="Q399" s="12" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
+      <c r="Q399" s="12" t="s">
+        <v>61</v>
       </c>
       <c r="R399" s="13" t="str">
         <f t="shared" ref="R399:R462" si="85">IF($P399="","",IF($Q399="Y",IFERROR(VLOOKUP($B399,$C$4:$D$13,2,FALSE()),0),0))</f>
@@ -41036,10 +41020,8 @@
         <f t="shared" si="84"/>
         <v/>
       </c>
-      <c r="Q445" s="12" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
+      <c r="Q445" s="12" t="s">
+        <v>61</v>
       </c>
       <c r="R445" s="13" t="str">
         <f t="shared" si="85"/>
@@ -41810,10 +41792,8 @@
         <f t="shared" si="84"/>
         <v/>
       </c>
-      <c r="Q455" s="12" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
+      <c r="Q455" s="12" t="s">
+        <v>61</v>
       </c>
       <c r="R455" s="13" t="str">
         <f t="shared" si="85"/>
@@ -42815,10 +42795,8 @@
         <f t="shared" si="97"/>
         <v/>
       </c>
-      <c r="Q468" s="12" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
+      <c r="Q468" s="12" t="s">
+        <v>61</v>
       </c>
       <c r="R468" s="13" t="str">
         <f t="shared" si="98"/>
@@ -42896,10 +42874,8 @@
         <f t="shared" si="97"/>
         <v/>
       </c>
-      <c r="Q469" s="12" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
+      <c r="Q469" s="12" t="s">
+        <v>61</v>
       </c>
       <c r="R469" s="13" t="str">
         <f t="shared" si="98"/>
@@ -43131,10 +43107,8 @@
         <f t="shared" si="97"/>
         <v/>
       </c>
-      <c r="Q472" s="12" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
+      <c r="Q472" s="12" t="s">
+        <v>61</v>
       </c>
       <c r="R472" s="13" t="str">
         <f t="shared" si="98"/>
@@ -45830,10 +45804,8 @@
         <f t="shared" si="97"/>
         <v/>
       </c>
-      <c r="Q507" s="12" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
+      <c r="Q507" s="12" t="s">
+        <v>61</v>
       </c>
       <c r="R507" s="13" t="str">
         <f t="shared" si="98"/>
@@ -49911,10 +49883,8 @@
         <f t="shared" si="110"/>
         <v/>
       </c>
-      <c r="Q560" s="12" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
+      <c r="Q560" s="12" t="s">
+        <v>61</v>
       </c>
       <c r="R560" s="13" t="str">
         <f t="shared" si="111"/>
@@ -50069,10 +50039,8 @@
         <f t="shared" si="110"/>
         <v/>
       </c>
-      <c r="Q562" s="12" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
+      <c r="Q562" s="12" t="s">
+        <v>61</v>
       </c>
       <c r="R562" s="13" t="str">
         <f t="shared" si="111"/>
@@ -50300,10 +50268,8 @@
         <f t="shared" si="110"/>
         <v/>
       </c>
-      <c r="Q565" s="12" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
+      <c r="Q565" s="12" t="s">
+        <v>61</v>
       </c>
       <c r="R565" s="13" t="str">
         <f t="shared" si="111"/>
@@ -50916,10 +50882,8 @@
         <f t="shared" si="110"/>
         <v/>
       </c>
-      <c r="Q573" s="12" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
+      <c r="Q573" s="12" t="s">
+        <v>61</v>
       </c>
       <c r="R573" s="13" t="str">
         <f t="shared" si="111"/>
@@ -51844,10 +51808,8 @@
         <f t="shared" si="110"/>
         <v/>
       </c>
-      <c r="Q585" s="12" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
+      <c r="Q585" s="12" t="s">
+        <v>61</v>
       </c>
       <c r="R585" s="13" t="str">
         <f t="shared" si="111"/>
@@ -56002,10 +55964,8 @@
         <f t="shared" si="123"/>
         <v/>
       </c>
-      <c r="Q639" s="12" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
+      <c r="Q639" s="12" t="s">
+        <v>61</v>
       </c>
       <c r="R639" s="13" t="str">
         <f t="shared" si="124"/>
@@ -58855,10 +58815,8 @@
         <f t="shared" si="136"/>
         <v/>
       </c>
-      <c r="Q676" s="12" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
+      <c r="Q676" s="12" t="s">
+        <v>61</v>
       </c>
       <c r="R676" s="13" t="str">
         <f t="shared" si="137"/>
@@ -59548,10 +59506,8 @@
         <f t="shared" si="136"/>
         <v/>
       </c>
-      <c r="Q685" s="12" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
+      <c r="Q685" s="12" t="s">
+        <v>61</v>
       </c>
       <c r="R685" s="13" t="str">
         <f t="shared" si="137"/>
@@ -63397,10 +63353,8 @@
         <f t="shared" si="149"/>
         <v/>
       </c>
-      <c r="Q735" s="12" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
+      <c r="Q735" s="12" t="s">
+        <v>61</v>
       </c>
       <c r="R735" s="13" t="str">
         <f t="shared" si="150"/>
@@ -65480,10 +65434,8 @@
         <f t="shared" si="149"/>
         <v/>
       </c>
-      <c r="Q762" s="12" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
+      <c r="Q762" s="12" t="s">
+        <v>61</v>
       </c>
       <c r="R762" s="13" t="str">
         <f t="shared" si="150"/>
@@ -66711,10 +66663,8 @@
         <f t="shared" si="149"/>
         <v/>
       </c>
-      <c r="Q778" s="12" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
+      <c r="Q778" s="12" t="s">
+        <v>61</v>
       </c>
       <c r="R778" s="13" t="str">
         <f t="shared" si="150"/>
@@ -66941,10 +66891,8 @@
         <f t="shared" si="149"/>
         <v/>
       </c>
-      <c r="Q781" s="12" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
+      <c r="Q781" s="12" t="s">
+        <v>61</v>
       </c>
       <c r="R781" s="13" t="str">
         <f t="shared" si="150"/>
@@ -69401,10 +69349,8 @@
         <f t="shared" si="164"/>
         <v/>
       </c>
-      <c r="Q813" s="12" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
+      <c r="Q813" s="12" t="s">
+        <v>61</v>
       </c>
       <c r="R813" s="13" t="str">
         <f t="shared" si="165"/>
@@ -71407,10 +71353,8 @@
         <f t="shared" si="164"/>
         <v/>
       </c>
-      <c r="Q839" s="12" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
+      <c r="Q839" s="12" t="s">
+        <v>61</v>
       </c>
       <c r="R839" s="13" t="str">
         <f t="shared" si="165"/>
@@ -72104,10 +72048,8 @@
         <f t="shared" si="178"/>
         <v/>
       </c>
-      <c r="Q848" s="12" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
+      <c r="Q848" s="12" t="s">
+        <v>61</v>
       </c>
       <c r="R848" s="13" t="str">
         <f t="shared" si="179"/>
@@ -72566,10 +72508,8 @@
         <f t="shared" si="178"/>
         <v/>
       </c>
-      <c r="Q854" s="12" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
+      <c r="Q854" s="12" t="s">
+        <v>61</v>
       </c>
       <c r="R854" s="13" t="str">
         <f t="shared" si="179"/>
@@ -74106,10 +74046,8 @@
         <f t="shared" si="178"/>
         <v/>
       </c>
-      <c r="Q874" s="12" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
+      <c r="Q874" s="12" t="s">
+        <v>61</v>
       </c>
       <c r="R874" s="13" t="str">
         <f t="shared" si="179"/>
@@ -74337,10 +74275,8 @@
         <f t="shared" si="178"/>
         <v/>
       </c>
-      <c r="Q877" s="12" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
+      <c r="Q877" s="12" t="s">
+        <v>61</v>
       </c>
       <c r="R877" s="13" t="str">
         <f t="shared" si="179"/>

</xml_diff>

<commit_message>
Use shared string for Hansol local currency flag
</commit_message>
<xml_diff>
--- a/fuel_cost_chungcheong.xlsx
+++ b/fuel_cost_chungcheong.xlsx
@@ -74970,10 +74970,8 @@
         <f t="shared" si="177"/>
         <v/>
       </c>
-      <c r="Q876" s="12" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
+      <c r="Q876" s="12" t="s">
+        <v>61</v>
       </c>
       <c r="R876" s="13" t="str">
         <f t="shared" si="178"/>

</xml_diff>

<commit_message>
Fix Hansol local currency cell to supported shared string
</commit_message>
<xml_diff>
--- a/fuel_cost_chungcheong.xlsx
+++ b/fuel_cost_chungcheong.xlsx
@@ -74970,10 +74970,8 @@
         <f t="shared" si="177"/>
         <v/>
       </c>
-      <c r="Q876" s="12" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
+      <c r="Q876" s="12" t="s">
+        <v>61</v>
       </c>
       <c r="R876" s="13" t="str">
         <f t="shared" si="178"/>

</xml_diff>

<commit_message>
Train PGO against corrected shared-string workbook
</commit_message>
<xml_diff>
--- a/fuel_cost_chungcheong.xlsx
+++ b/fuel_cost_chungcheong.xlsx
@@ -74970,10 +74970,8 @@
         <f t="shared" si="177"/>
         <v/>
       </c>
-      <c r="Q876" s="12" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
+      <c r="Q876" s="12" t="s">
+        <v>61</v>
       </c>
       <c r="R876" s="13" t="str">
         <f t="shared" si="178"/>

</xml_diff>